<commit_message>
feat(finops): usa la cobertura ACT medida (92,2 %) y calcula el % de equilibrio
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cloud/finops_model.xlsx
+++ b/docs/cloud/finops_model.xlsx
@@ -210,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -247,6 +247,7 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -347,7 +348,7 @@
   <commentList>
     <comment ref="C16" authorId="0" shapeId="0">
       <text>
-        <t>Coordinador: reemplazar por la cobertura ACT medida en test (reporte del modelo).</t>
+        <t>Medido en COIL-100 (protocolo A). En planta real debe re-medirse en el piloto.</t>
       </text>
     </comment>
   </commentList>
@@ -1068,7 +1069,7 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>0.95</v>
+        <v>0.922</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1077,12 +1078,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Medido</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>PLACEHOLDER sin evidencia: reemplazar por la cobertura ACT medida en test (docs/report). Ver Sensibilidad 80-99%</t>
+          <t>Cobertura ACT medida en test, protocolo A, receta classic-logreg-v1 (docs/report/results.json): 92,2 % con 0,21 % de error entre ACT. Con desconocidos mezclados (D variante) baja a 77,0 %. Planta real: validar en piloto. Ver Sensibilidad</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -8056,7 +8057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -8517,36 +8518,59 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Lectura rápida:</t>
-        </is>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>% automatizado de equilibrio (ahorro = 0)</t>
+        </is>
+      </c>
+      <c r="B24" s="30">
+        <f>-(actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))/((actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))-(actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)))</f>
+        <v/>
+      </c>
+      <c r="C24" s="30">
+        <f>-(actual_mes_co-((aws_total_mes-aws_img_mes+aws_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))/((actual_mes_co-((aws_total_mes-aws_img_mes+aws_img_mes*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))-(actual_mes_co-((aws_total_mes-aws_img_mes+aws_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)))</f>
+        <v/>
+      </c>
+      <c r="D24" s="30">
+        <f>-(actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))/((actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))-(actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)))</f>
+        <v/>
+      </c>
+      <c r="E24" s="30">
+        <f>-(actual_mes_es-((aws_total_mes_ue-aws_img_mes_ue+aws_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))/((actual_mes_es-((aws_total_mes_ue-aws_img_mes_ue+aws_img_mes_ue*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))-(actual_mes_es-((aws_total_mes_ue-aws_img_mes_ue+aws_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)))</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• El ahorro viene de retirar 3 turnos de operador por estación; la nube es una fracción pequeña del costo laboral evitado.</t>
+          <t>Lectura rápida:</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• El factor que más mueve el resultado es % automatizado (cola de revisión) y el costo laboral local, no el proveedor de nube.</t>
+          <t>• El ahorro viene de retirar 3 turnos de operador por estación; la nube es una fracción pequeña del costo laboral evitado.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• Con 1 estación en Colombia el payback es largo: el CAPEX de implementación por planta pesa mucho (ver Sensibilidad).</t>
+          <t>• El factor que más mueve el resultado es % automatizado (cola de revisión) y el costo laboral local, no el proveedor de nube.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
+        <is>
+          <t>• Con 1 estación en Colombia el payback es largo: el CAPEX de implementación por planta pesa mucho (ver Sensibilidad).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>• Ningún número de esta hoja está hardcodeado: todo sale de Supuestos, Operación actual, Azure y AWS.</t>
         </is>
@@ -8566,7 +8590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8601,7 +8625,7 @@
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
-          <t>1) % automatizado (estaciones de Supuestos) — Azure. El almacenamiento de imágenes también escala con el %.</t>
+          <t>1) % automatizado (estaciones de Supuestos) — Azure. 92,2% = medido (protocolo A); 77,0% = medido con objetos desconocidos mezclados (variante D). El almacenamiento de imágenes también escala con el %.</t>
         </is>
       </c>
     </row>
@@ -8643,343 +8667,374 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="n">
+      <c r="A6" s="31" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="B6" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C6" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A6)+$A6*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D6" s="33">
+        <f>IF(C6&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C6,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E6" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F6" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A6)+$A6*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G6" s="33">
+        <f>IF(F6&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F6,"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="n">
         <v>0.8</v>
       </c>
-      <c r="B6" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_co</f>
-        <v/>
-      </c>
-      <c r="C6" s="31">
-        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A6)+$A6*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+B6+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
-        <v/>
-      </c>
-      <c r="D6" s="32">
-        <f>IF(C6&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C6,"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E6" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_es</f>
-        <v/>
-      </c>
-      <c r="F6" s="31">
-        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A6)+$A6*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+E6+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
-        <v/>
-      </c>
-      <c r="G6" s="32">
-        <f>IF(F6&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F6,"No recupera")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="n">
+      <c r="B7" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C7" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A7)+$A7*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D7" s="33">
+        <f>IF(C7&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C7,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E7" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F7" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A7)+$A7*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G7" s="33">
+        <f>IF(F7&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F7,"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="n">
         <v>0.9</v>
       </c>
-      <c r="B7" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_co</f>
-        <v/>
-      </c>
-      <c r="C7" s="31">
-        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A7)+$A7*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+B7+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
-        <v/>
-      </c>
-      <c r="D7" s="32">
-        <f>IF(C7&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C7,"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E7" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_es</f>
-        <v/>
-      </c>
-      <c r="F7" s="31">
-        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A7)+$A7*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+E7+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
-        <v/>
-      </c>
-      <c r="G7" s="32">
-        <f>IF(F7&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F7,"No recupera")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="n">
+      <c r="B8" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C8" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A8)+$A8*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D8" s="33">
+        <f>IF(C8&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C8,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E8" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F8" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A8)+$A8*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G8" s="33">
+        <f>IF(F8&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F8,"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="n">
+        <v>0.922</v>
+      </c>
+      <c r="B9" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C9" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A9)+$A9*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D9" s="33">
+        <f>IF(C9&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C9,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E9" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F9" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A9)+$A9*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G9" s="33">
+        <f>IF(F9&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F9,"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="n">
         <v>0.95</v>
       </c>
-      <c r="B8" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_co</f>
-        <v/>
-      </c>
-      <c r="C8" s="31">
-        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A8)+$A8*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+B8+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
-        <v/>
-      </c>
-      <c r="D8" s="32">
-        <f>IF(C8&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C8,"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E8" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_es</f>
-        <v/>
-      </c>
-      <c r="F8" s="31">
-        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A8)+$A8*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+E8+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
-        <v/>
-      </c>
-      <c r="G8" s="32">
-        <f>IF(F8&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F8,"No recupera")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="n">
+      <c r="B10" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C10" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A10)+$A10*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D10" s="33">
+        <f>IF(C10&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C10,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E10" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F10" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A10)+$A10*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G10" s="33">
+        <f>IF(F10&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F10,"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="n">
         <v>0.99</v>
       </c>
-      <c r="B9" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_co</f>
-        <v/>
-      </c>
-      <c r="C9" s="31">
-        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A9)+$A9*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+B9+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
-        <v/>
-      </c>
-      <c r="D9" s="32">
-        <f>IF(C9&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C9,"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E9" s="31">
-        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_es</f>
-        <v/>
-      </c>
-      <c r="F9" s="31">
-        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A9)+$A9*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+E9+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
-        <v/>
-      </c>
-      <c r="G9" s="32">
-        <f>IF(F9&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F9,"No recupera")</f>
+      <c r="B11" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C11" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A11)+$A11*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D11" s="33">
+        <f>IF(C11&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C11,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E11" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F11" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A11)+$A11*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G11" s="33">
+        <f>IF(F11&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F11,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
         <is>
+          <t>Equilibrio (ahorro = 0)</t>
+        </is>
+      </c>
+      <c r="C12" s="30">
+        <f>-(actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))/((actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))-(actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)))</f>
+        <v/>
+      </c>
+      <c r="F12" s="30">
+        <f>-(actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))/((actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))-(actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
           <t>2) Estaciones por planta (% automatizado de Supuestos) — Azure</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Estaciones</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Costo actual CO</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Costo nuevo CO</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Payback CO (meses)</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Costo actual ES</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Costo nuevo ES</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Payback ES (meses)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="33" t="n">
+    <row r="16">
+      <c r="A16" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="31">
-        <f>actual_estacion_co*$A14*plantas</f>
-        <v/>
-      </c>
-      <c r="C14" s="31">
-        <f>(azure_fijo_mes+azure_por_estacion_mes*$A14+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A14)*dias_mes)*plantas+$A14*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="D14" s="32">
-        <f>IF(B14&gt;C14,($A14*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B14-C14),"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E14" s="31">
-        <f>actual_estacion_es*$A14*plantas</f>
-        <v/>
-      </c>
-      <c r="F14" s="31">
-        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A14+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A14)*dias_mes)*plantas+$A14*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="G14" s="32">
-        <f>IF(E14&gt;F14,($A14*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E14-F14),"No recupera")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="33" t="n">
+      <c r="B16" s="32">
+        <f>actual_estacion_co*$A16*plantas</f>
+        <v/>
+      </c>
+      <c r="C16" s="32">
+        <f>(azure_fijo_mes+azure_por_estacion_mes*$A16+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A16)*dias_mes)*plantas+$A16*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="D16" s="33">
+        <f>IF(B16&gt;C16,($A16*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B16-C16),"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E16" s="32">
+        <f>actual_estacion_es*$A16*plantas</f>
+        <v/>
+      </c>
+      <c r="F16" s="32">
+        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A16+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A16)*dias_mes)*plantas+$A16*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="G16" s="33">
+        <f>IF(E16&gt;F16,($A16*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E16-F16),"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="B15" s="31">
-        <f>actual_estacion_co*$A15*plantas</f>
-        <v/>
-      </c>
-      <c r="C15" s="31">
-        <f>(azure_fijo_mes+azure_por_estacion_mes*$A15+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A15)*dias_mes)*plantas+$A15*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="D15" s="32">
-        <f>IF(B15&gt;C15,($A15*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B15-C15),"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E15" s="31">
-        <f>actual_estacion_es*$A15*plantas</f>
-        <v/>
-      </c>
-      <c r="F15" s="31">
-        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A15+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A15)*dias_mes)*plantas+$A15*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="G15" s="32">
-        <f>IF(E15&gt;F15,($A15*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E15-F15),"No recupera")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33" t="n">
+      <c r="B17" s="32">
+        <f>actual_estacion_co*$A17*plantas</f>
+        <v/>
+      </c>
+      <c r="C17" s="32">
+        <f>(azure_fijo_mes+azure_por_estacion_mes*$A17+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A17)*dias_mes)*plantas+$A17*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="D17" s="33">
+        <f>IF(B17&gt;C17,($A17*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B17-C17),"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E17" s="32">
+        <f>actual_estacion_es*$A17*plantas</f>
+        <v/>
+      </c>
+      <c r="F17" s="32">
+        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A17+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A17)*dias_mes)*plantas+$A17*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="G17" s="33">
+        <f>IF(E17&gt;F17,($A17*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E17-F17),"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="B16" s="31">
-        <f>actual_estacion_co*$A16*plantas</f>
-        <v/>
-      </c>
-      <c r="C16" s="31">
-        <f>(azure_fijo_mes+azure_por_estacion_mes*$A16+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A16)*dias_mes)*plantas+$A16*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="D16" s="32">
-        <f>IF(B16&gt;C16,($A16*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B16-C16),"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E16" s="31">
-        <f>actual_estacion_es*$A16*plantas</f>
-        <v/>
-      </c>
-      <c r="F16" s="31">
-        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A16+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A16)*dias_mes)*plantas+$A16*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="G16" s="32">
-        <f>IF(E16&gt;F16,($A16*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E16-F16),"No recupera")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="B18" s="32">
+        <f>actual_estacion_co*$A18*plantas</f>
+        <v/>
+      </c>
+      <c r="C18" s="32">
+        <f>(azure_fijo_mes+azure_por_estacion_mes*$A18+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A18)*dias_mes)*plantas+$A18*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="D18" s="33">
+        <f>IF(B18&gt;C18,($A18*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B18-C18),"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E18" s="32">
+        <f>actual_estacion_es*$A18*plantas</f>
+        <v/>
+      </c>
+      <c r="F18" s="32">
+        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A18+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A18)*dias_mes)*plantas+$A18*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="G18" s="33">
+        <f>IF(E18&gt;F18,($A18*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E18-F18),"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>3) Volumen del asistente: costo LLM mensual por planta (precios EE. UU.)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Conversaciones/día</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Azure LLM (USD/mes)</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>AWS LLM (USD/mes)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Azure si todo va a gpt-4.1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Peso LLM en nube Azure</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="33" t="n">
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="31">
-        <f>azure_llm_por_conv*$A21*dias_mes</f>
-        <v/>
-      </c>
-      <c r="C21" s="31">
-        <f>aws_llm_por_conv*$A21*dias_mes</f>
-        <v/>
-      </c>
-      <c r="D21" s="31">
-        <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A21*dias_mes</f>
-        <v/>
-      </c>
-      <c r="E21" s="29">
-        <f>B21/(azure_fijo_mes+azure_estacion_total_mes+B21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33" t="n">
-        <v>60</v>
-      </c>
-      <c r="B22" s="31">
-        <f>azure_llm_por_conv*$A22*dias_mes</f>
-        <v/>
-      </c>
-      <c r="C22" s="31">
-        <f>aws_llm_por_conv*$A22*dias_mes</f>
-        <v/>
-      </c>
-      <c r="D22" s="31">
-        <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A22*dias_mes</f>
-        <v/>
-      </c>
-      <c r="E22" s="29">
-        <f>B22/(azure_fijo_mes+azure_estacion_total_mes+B22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="B23" s="31">
+      <c r="B23" s="32">
         <f>azure_llm_por_conv*$A23*dias_mes</f>
         <v/>
       </c>
-      <c r="C23" s="31">
+      <c r="C23" s="32">
         <f>aws_llm_por_conv*$A23*dias_mes</f>
         <v/>
       </c>
-      <c r="D23" s="31">
+      <c r="D23" s="32">
         <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A23*dias_mes</f>
         <v/>
       </c>
@@ -8989,18 +9044,18 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="33" t="n">
-        <v>1000</v>
-      </c>
-      <c r="B24" s="31">
+      <c r="A24" s="34" t="n">
+        <v>60</v>
+      </c>
+      <c r="B24" s="32">
         <f>azure_llm_por_conv*$A24*dias_mes</f>
         <v/>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="32">
         <f>aws_llm_por_conv*$A24*dias_mes</f>
         <v/>
       </c>
-      <c r="D24" s="31">
+      <c r="D24" s="32">
         <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A24*dias_mes</f>
         <v/>
       </c>
@@ -9009,8 +9064,50 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="34" t="n">
+        <v>200</v>
+      </c>
+      <c r="B25" s="32">
+        <f>azure_llm_por_conv*$A25*dias_mes</f>
+        <v/>
+      </c>
+      <c r="C25" s="32">
+        <f>aws_llm_por_conv*$A25*dias_mes</f>
+        <v/>
+      </c>
+      <c r="D25" s="32">
+        <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A25*dias_mes</f>
+        <v/>
+      </c>
+      <c r="E25" s="29">
+        <f>B25/(azure_fijo_mes+azure_estacion_total_mes+B25)</f>
+        <v/>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="34" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B26" s="32">
+        <f>azure_llm_por_conv*$A26*dias_mes</f>
+        <v/>
+      </c>
+      <c r="C26" s="32">
+        <f>aws_llm_por_conv*$A26*dias_mes</f>
+        <v/>
+      </c>
+      <c r="D26" s="32">
+        <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A26*dias_mes</f>
+        <v/>
+      </c>
+      <c r="E26" s="29">
+        <f>B26/(azure_fijo_mes+azure_estacion_total_mes+B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>La columna 'todo a gpt-4.1' usa las celdas de precio gpt-4.1 de la hoja Azure (rangos azure_big_*).</t>
         </is>
@@ -9152,7 +9249,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I5" s="34" t="inlineStr">
+      <c r="I5" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard vCPU Active Usage'</t>
         </is>
@@ -9197,7 +9294,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I6" s="34" t="inlineStr">
+      <c r="I6" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard vCPU Active Usage'</t>
         </is>
@@ -9242,7 +9339,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I7" s="34" t="inlineStr">
+      <c r="I7" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard Memory Active Usage'</t>
         </is>
@@ -9287,7 +9384,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I8" s="34" t="inlineStr">
+      <c r="I8" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard Memory Active Usage'</t>
         </is>
@@ -9332,7 +9429,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I9" s="34" t="inlineStr">
+      <c r="I9" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Environment Private Endpoint'</t>
         </is>
@@ -9377,7 +9474,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I10" s="34" t="inlineStr">
+      <c r="I10" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Environment Private Endpoint'</t>
         </is>
@@ -9422,7 +9519,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I11" s="34" t="inlineStr">
+      <c r="I11" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Container Registry' and meterName eq 'Basic Registry Unit'</t>
         </is>
@@ -9467,7 +9564,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I12" s="34" t="inlineStr">
+      <c r="I12" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Container Registry' and meterName eq 'Basic Registry Unit'</t>
         </is>
@@ -9512,7 +9609,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I13" s="34" t="inlineStr">
+      <c r="I13" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Virtual Machines' and armSkuName eq 'Standard_D4s_v3' and meterName eq 'D4s v3'</t>
         </is>
@@ -9557,7 +9654,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I14" s="34" t="inlineStr">
+      <c r="I14" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Virtual Machines' and armSkuName eq 'Standard_D4s_v3' and meterName eq 'D4s v3'</t>
         </is>
@@ -9602,7 +9699,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I15" s="34" t="inlineStr">
+      <c r="I15" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flexible Server General Purpose Ddsv5 Series Compute' and skuName eq '2 vCore'</t>
         </is>
@@ -9647,7 +9744,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I16" s="34" t="inlineStr">
+      <c r="I16" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flexible Server General Purpose Ddsv5 Series Compute' and skuName eq '2 vCore'</t>
         </is>
@@ -9692,7 +9789,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I17" s="34" t="inlineStr">
+      <c r="I17" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flex Server Storage' and meterName eq 'Storage Data Stored'</t>
         </is>
@@ -9737,7 +9834,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I18" s="34" t="inlineStr">
+      <c r="I18" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flex Server Storage' and meterName eq 'Storage Data Stored'</t>
         </is>
@@ -9782,7 +9879,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I19" s="34" t="inlineStr">
+      <c r="I19" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Cognitive Search' and meterName eq 'Basic Unit'</t>
         </is>
@@ -9827,7 +9924,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I20" s="34" t="inlineStr">
+      <c r="I20" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Cognitive Search' and meterName eq 'Basic Unit'</t>
         </is>
@@ -9872,7 +9969,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I21" s="34" t="inlineStr">
+      <c r="I21" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot LRS Data Stored'</t>
         </is>
@@ -9917,7 +10014,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I22" s="34" t="inlineStr">
+      <c r="I22" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot LRS Data Stored'</t>
         </is>
@@ -9962,7 +10059,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I23" s="34" t="inlineStr">
+      <c r="I23" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Cool LRS Data Stored'</t>
         </is>
@@ -10007,7 +10104,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I24" s="34" t="inlineStr">
+      <c r="I24" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Cool LRS Data Stored'</t>
         </is>
@@ -10052,7 +10149,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I25" s="34" t="inlineStr">
+      <c r="I25" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Archive LRS Data Stored'</t>
         </is>
@@ -10097,7 +10194,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I26" s="34" t="inlineStr">
+      <c r="I26" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Archive LRS Data Stored'</t>
         </is>
@@ -10142,7 +10239,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I27" s="34" t="inlineStr">
+      <c r="I27" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot ZRS Data Stored'</t>
         </is>
@@ -10187,7 +10284,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I28" s="34" t="inlineStr">
+      <c r="I28" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot ZRS Data Stored'</t>
         </is>
@@ -10232,7 +10329,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I29" s="34" t="inlineStr">
+      <c r="I29" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'IoT Hub' and meterName eq 'S1 Unit'</t>
         </is>
@@ -10277,7 +10374,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I30" s="34" t="inlineStr">
+      <c r="I30" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'westeurope' and priceType eq 'Consumption' and serviceName eq 'IoT Hub' and meterName eq 'S1 Unit'</t>
         </is>
@@ -10322,7 +10419,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I31" s="34" t="inlineStr">
+      <c r="I31" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Servers' and meterName eq 'Standard P2 Node'</t>
         </is>
@@ -10367,7 +10464,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I32" s="34" t="inlineStr">
+      <c r="I32" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Servers' and meterName eq 'Standard P2 Node'</t>
         </is>
@@ -10412,7 +10509,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I33" s="34" t="inlineStr">
+      <c r="I33" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Key Vault' and skuName eq 'Standard' and meterName eq 'Operations'</t>
         </is>
@@ -10457,7 +10554,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I34" s="34" t="inlineStr">
+      <c r="I34" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Key Vault' and skuName eq 'Standard' and meterName eq 'Operations'</t>
         </is>
@@ -10502,7 +10599,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I35" s="34" t="inlineStr">
+      <c r="I35" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Log Analytics' and meterName eq 'Analytics Logs Data Ingestion'</t>
         </is>
@@ -10547,7 +10644,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I36" s="34" t="inlineStr">
+      <c r="I36" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Log Analytics' and meterName eq 'Analytics Logs Data Ingestion'</t>
         </is>
@@ -10592,7 +10689,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I37" s="34" t="inlineStr">
+      <c r="I37" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Containers' and meterName eq 'Standard Images'</t>
         </is>
@@ -10637,7 +10734,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I38" s="34" t="inlineStr">
+      <c r="I38" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Containers' and meterName eq 'Standard Images'</t>
         </is>
@@ -10682,7 +10779,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I39" s="34" t="inlineStr">
+      <c r="I39" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'text-embedding-3-small-glbl Tokens'</t>
         </is>
@@ -10727,7 +10824,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I40" s="34" t="inlineStr">
+      <c r="I40" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'text-embedding-3-small-glbl Tokens'</t>
         </is>
@@ -10772,7 +10869,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I41" s="34" t="inlineStr">
+      <c r="I41" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Inp Data Zone Tokens'</t>
         </is>
@@ -10817,7 +10914,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I42" s="34" t="inlineStr">
+      <c r="I42" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Inp Data Zone Tokens'</t>
         </is>
@@ -10862,7 +10959,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I43" s="34" t="inlineStr">
+      <c r="I43" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini cached Inp DZone Tokens'</t>
         </is>
@@ -10907,7 +11004,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I44" s="34" t="inlineStr">
+      <c r="I44" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini cached Inp DZone Tokens'</t>
         </is>
@@ -10952,7 +11049,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I45" s="34" t="inlineStr">
+      <c r="I45" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Outp Data Zone Tokens'</t>
         </is>
@@ -10997,7 +11094,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I46" s="34" t="inlineStr">
+      <c r="I46" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Outp Data Zone Tokens'</t>
         </is>
@@ -11042,7 +11139,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I47" s="34" t="inlineStr">
+      <c r="I47" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Inp Data Zone Tokens'</t>
         </is>
@@ -11087,7 +11184,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I48" s="34" t="inlineStr">
+      <c r="I48" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Inp Data Zone Tokens'</t>
         </is>
@@ -11132,7 +11229,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I49" s="34" t="inlineStr">
+      <c r="I49" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 cached Inp Data Zone Tokens'</t>
         </is>
@@ -11177,7 +11274,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I50" s="34" t="inlineStr">
+      <c r="I50" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 cached Inp Data Zone Tokens'</t>
         </is>
@@ -11222,7 +11319,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I51" s="34" t="inlineStr">
+      <c r="I51" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Outp Data Zone Tokens'</t>
         </is>
@@ -11267,7 +11364,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I52" s="34" t="inlineStr">
+      <c r="I52" s="35" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Outp Data Zone Tokens'</t>
         </is>
@@ -11312,7 +11409,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I53" s="34" t="inlineStr">
+      <c r="I53" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/us-east-1/index.json</t>
         </is>
@@ -11357,7 +11454,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I54" s="34" t="inlineStr">
+      <c r="I54" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/eu-south-2/index.json</t>
         </is>
@@ -11402,7 +11499,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I55" s="34" t="inlineStr">
+      <c r="I55" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/us-east-1/index.json</t>
         </is>
@@ -11447,7 +11544,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I56" s="34" t="inlineStr">
+      <c r="I56" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/eu-south-2/index.json</t>
         </is>
@@ -11492,7 +11589,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I57" s="34" t="inlineStr">
+      <c r="I57" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/us-east-1/index.json</t>
         </is>
@@ -11537,7 +11634,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I58" s="34" t="inlineStr">
+      <c r="I58" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/eu-south-2/index.json</t>
         </is>
@@ -11582,7 +11679,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I59" s="34" t="inlineStr">
+      <c r="I59" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/us-east-1/index.json</t>
         </is>
@@ -11627,7 +11724,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I60" s="34" t="inlineStr">
+      <c r="I60" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/eu-south-2/index.json</t>
         </is>
@@ -11672,7 +11769,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I61" s="34" t="inlineStr">
+      <c r="I61" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonVPC/current/us-east-1/index.json</t>
         </is>
@@ -11717,7 +11814,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I62" s="34" t="inlineStr">
+      <c r="I62" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonVPC/current/eu-south-2/index.json</t>
         </is>
@@ -11762,7 +11859,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I63" s="34" t="inlineStr">
+      <c r="I63" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECR/current/us-east-1/index.json</t>
         </is>
@@ -11807,7 +11904,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I64" s="34" t="inlineStr">
+      <c r="I64" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECR/current/eu-south-2/index.json</t>
         </is>
@@ -11852,7 +11949,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I65" s="34" t="inlineStr">
+      <c r="I65" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonSageMaker/current/us-east-1/index.json</t>
         </is>
@@ -11897,7 +11994,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I66" s="34" t="inlineStr">
+      <c r="I66" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonSageMaker/current/eu-south-2/index.json</t>
         </is>
@@ -11942,7 +12039,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I67" s="34" t="inlineStr">
+      <c r="I67" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/us-east-1/index.json</t>
         </is>
@@ -11987,7 +12084,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I68" s="34" t="inlineStr">
+      <c r="I68" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/eu-south-2/index.json</t>
         </is>
@@ -12032,7 +12129,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I69" s="34" t="inlineStr">
+      <c r="I69" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/us-east-1/index.json</t>
         </is>
@@ -12077,7 +12174,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I70" s="34" t="inlineStr">
+      <c r="I70" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/eu-south-2/index.json</t>
         </is>
@@ -12122,7 +12219,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I71" s="34" t="inlineStr">
+      <c r="I71" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/us-east-1/index.json</t>
         </is>
@@ -12167,7 +12264,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I72" s="34" t="inlineStr">
+      <c r="I72" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/eu-south-2/index.json</t>
         </is>
@@ -12212,7 +12309,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I73" s="34" t="inlineStr">
+      <c r="I73" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/us-east-1/index.json</t>
         </is>
@@ -12257,7 +12354,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I74" s="34" t="inlineStr">
+      <c r="I74" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/eu-south-2/index.json</t>
         </is>
@@ -12302,7 +12399,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I75" s="34" t="inlineStr">
+      <c r="I75" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3GlacierDeepArchive/current/us-east-1/index.json</t>
         </is>
@@ -12347,7 +12444,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I76" s="34" t="inlineStr">
+      <c r="I76" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3GlacierDeepArchive/current/eu-south-2/index.json</t>
         </is>
@@ -12392,7 +12489,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I77" s="34" t="inlineStr">
+      <c r="I77" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/us-east-1/index.json</t>
         </is>
@@ -12437,7 +12534,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I78" s="34" t="inlineStr">
+      <c r="I78" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/eu-south-2/index.json</t>
         </is>
@@ -12482,7 +12579,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I79" s="34" t="inlineStr">
+      <c r="I79" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/us-east-1/index.json</t>
         </is>
@@ -12527,7 +12624,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I80" s="34" t="inlineStr">
+      <c r="I80" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/eu-south-2/index.json</t>
         </is>
@@ -12572,7 +12669,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I81" s="34" t="inlineStr">
+      <c r="I81" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSGreengrass/current/us-east-1/index.json</t>
         </is>
@@ -12617,7 +12714,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I82" s="34" t="inlineStr">
+      <c r="I82" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSGreengrass/current/eu-south-2/index.json</t>
         </is>
@@ -12662,7 +12759,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I83" s="34" t="inlineStr">
+      <c r="I83" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSSecretsManager/current/us-east-1/index.json</t>
         </is>
@@ -12707,7 +12804,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I84" s="34" t="inlineStr">
+      <c r="I84" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSSecretsManager/current/eu-south-2/index.json</t>
         </is>
@@ -12752,7 +12849,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I85" s="34" t="inlineStr">
+      <c r="I85" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonCloudWatch/current/us-east-1/index.json</t>
         </is>
@@ -12797,7 +12894,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I86" s="34" t="inlineStr">
+      <c r="I86" s="35" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonCloudWatch/current/eu-south-2/index.json</t>
         </is>

</xml_diff>

<commit_message>
feat(finops): actualiza costos con la cobertura medida de vision-1.0.1 (90,3 %)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cloud/finops_model.xlsx
+++ b/docs/cloud/finops_model.xlsx
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>0.922</v>
+        <v>0.903</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Cobertura ACT medida en test, protocolo A, receta classic-logreg-v1 (docs/report/results.json): 92,2 % con 0,21 % de error entre ACT. Con desconocidos mezclados (D variante) baja a 77,0 %. Planta real: validar en piloto. Ver Sensibilidad</t>
+          <t>Cobertura ACT medida en test, protocolo A, vision-1.0.1 (docs/report/results.json): 90,3 % con 0,09 % de error entre ACT (IC95 0,03-0,27 %). Con desconocidos mezclados (D variante) baja a 73,7-74,9 %. Planta real: re-medir en piloto. Ver Sensibilidad</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -8590,7 +8590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8625,7 +8625,7 @@
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
-          <t>1) % automatizado (estaciones de Supuestos) — Azure. 92,2% = medido (protocolo A); 77,0% = medido con objetos desconocidos mezclados (variante D). El almacenamiento de imágenes también escala con el %.</t>
+          <t>1) % automatizado (estaciones de Supuestos) — Azure. 90,3% = medido (vision-1.0.1, protocolo A); 73,7-74,9% = medido con objetos desconocidos mezclados (variante D). El almacenamiento de imágenes también escala con el %.</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
     </row>
     <row r="6">
       <c r="A6" s="31" t="n">
-        <v>0.77</v>
+        <v>0.737</v>
       </c>
       <c r="B6" s="32">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_co</f>
@@ -8697,7 +8697,7 @@
     </row>
     <row r="7">
       <c r="A7" s="31" t="n">
-        <v>0.8</v>
+        <v>0.749</v>
       </c>
       <c r="B7" s="32">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_co</f>
@@ -8726,7 +8726,7 @@
     </row>
     <row r="8">
       <c r="A8" s="31" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="B8" s="32">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_co</f>
@@ -8755,7 +8755,7 @@
     </row>
     <row r="9">
       <c r="A9" s="31" t="n">
-        <v>0.922</v>
+        <v>0.9</v>
       </c>
       <c r="B9" s="32">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_co</f>
@@ -8784,7 +8784,7 @@
     </row>
     <row r="10">
       <c r="A10" s="31" t="n">
-        <v>0.95</v>
+        <v>0.903</v>
       </c>
       <c r="B10" s="32">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_co</f>
@@ -8813,7 +8813,7 @@
     </row>
     <row r="11">
       <c r="A11" s="31" t="n">
-        <v>0.99</v>
+        <v>0.95</v>
       </c>
       <c r="B11" s="32">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_co</f>
@@ -8841,96 +8841,96 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="31" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="B12" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_co</f>
+        <v/>
+      </c>
+      <c r="C12" s="32">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A12)+$A12*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D12" s="33">
+        <f>IF(C12&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C12,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E12" s="32">
+        <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_es</f>
+        <v/>
+      </c>
+      <c r="F12" s="32">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A12)+$A12*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="G12" s="33">
+        <f>IF(F12&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F12,"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Equilibrio (ahorro = 0)</t>
         </is>
       </c>
-      <c r="C12" s="30">
+      <c r="C13" s="30">
         <f>-(actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))/((actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co))-(actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)))</f>
         <v/>
       </c>
-      <c r="F12" s="30">
+      <c r="F13" s="30">
         <f>-(actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))/((actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-1)+1*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-1)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es))-(actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-0)+0*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-0)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)))</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>2) Estaciones por planta (% automatizado de Supuestos) — Azure</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Estaciones</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Costo actual CO</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Costo nuevo CO</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Payback CO (meses)</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Costo actual ES</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Costo nuevo ES</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Payback ES (meses)</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="32">
-        <f>actual_estacion_co*$A16*plantas</f>
-        <v/>
-      </c>
-      <c r="C16" s="32">
-        <f>(azure_fijo_mes+azure_por_estacion_mes*$A16+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A16)*dias_mes)*plantas+$A16*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="D16" s="33">
-        <f>IF(B16&gt;C16,($A16*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B16-C16),"No recupera")</f>
-        <v/>
-      </c>
-      <c r="E16" s="32">
-        <f>actual_estacion_es*$A16*plantas</f>
-        <v/>
-      </c>
-      <c r="F16" s="32">
-        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A16+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A16)*dias_mes)*plantas+$A16*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
-        <v/>
-      </c>
-      <c r="G16" s="33">
-        <f>IF(E16&gt;F16,($A16*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E16-F16),"No recupera")</f>
-        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B17" s="32">
         <f>actual_estacion_co*$A17*plantas</f>
@@ -8959,7 +8959,7 @@
     </row>
     <row r="18">
       <c r="A18" s="34" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B18" s="32">
         <f>actual_estacion_co*$A18*plantas</f>
@@ -8986,66 +8986,74 @@
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="22" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B19" s="32">
+        <f>actual_estacion_co*$A19*plantas</f>
+        <v/>
+      </c>
+      <c r="C19" s="32">
+        <f>(azure_fijo_mes+azure_por_estacion_mes*$A19+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A19)*dias_mes)*plantas+$A19*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="D19" s="33">
+        <f>IF(B19&gt;C19,($A19*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B19-C19),"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E19" s="32">
+        <f>actual_estacion_es*$A19*plantas</f>
+        <v/>
+      </c>
+      <c r="F19" s="32">
+        <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A19+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A19)*dias_mes)*plantas+$A19*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
+        <v/>
+      </c>
+      <c r="G19" s="33">
+        <f>IF(E19&gt;F19,($A19*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E19-F19),"No recupera")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>3) Volumen del asistente: costo LLM mensual por planta (precios EE. UU.)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Conversaciones/día</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Azure LLM (USD/mes)</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>AWS LLM (USD/mes)</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Azure si todo va a gpt-4.1</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Peso LLM en nube Azure</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="32">
-        <f>azure_llm_por_conv*$A23*dias_mes</f>
-        <v/>
-      </c>
-      <c r="C23" s="32">
-        <f>aws_llm_por_conv*$A23*dias_mes</f>
-        <v/>
-      </c>
-      <c r="D23" s="32">
-        <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A23*dias_mes</f>
-        <v/>
-      </c>
-      <c r="E23" s="29">
-        <f>B23/(azure_fijo_mes+azure_estacion_total_mes+B23)</f>
-        <v/>
-      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="34" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="B24" s="32">
         <f>azure_llm_por_conv*$A24*dias_mes</f>
@@ -9066,7 +9074,7 @@
     </row>
     <row r="25">
       <c r="A25" s="34" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="B25" s="32">
         <f>azure_llm_por_conv*$A25*dias_mes</f>
@@ -9087,7 +9095,7 @@
     </row>
     <row r="26">
       <c r="A26" s="34" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="B26" s="32">
         <f>azure_llm_por_conv*$A26*dias_mes</f>
@@ -9106,8 +9114,29 @@
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="34" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B27" s="32">
+        <f>azure_llm_por_conv*$A27*dias_mes</f>
+        <v/>
+      </c>
+      <c r="C27" s="32">
+        <f>aws_llm_por_conv*$A27*dias_mes</f>
+        <v/>
+      </c>
+      <c r="D27" s="32">
+        <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A27*dias_mes</f>
+        <v/>
+      </c>
+      <c r="E27" s="29">
+        <f>B27/(azure_fijo_mes+azure_estacion_total_mes+B27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>La columna 'todo a gpt-4.1' usa las celdas de precio gpt-4.1 de la hoja Azure (rangos azure_big_*).</t>
         </is>

</xml_diff>

<commit_message>
docs(finops): caso de negocio como rango con escenario pesimista medido (73,7 %)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cloud/finops_model.xlsx
+++ b/docs/cloud/finops_model.xlsx
@@ -26,52 +26,53 @@
     <definedName name="factor_cobertura">'Supuestos'!$C$13</definedName>
     <definedName name="throughput_obj_h">'Supuestos'!$C$14</definedName>
     <definedName name="pct_automatizado">'Supuestos'!$C$16</definedName>
-    <definedName name="min_caso_revision">'Supuestos'!$C$17</definedName>
-    <definedName name="fraccion_atencion">'Supuestos'!$C$18</definedName>
-    <definedName name="salario_co_cop">'Supuestos'!$C$20</definedName>
-    <definedName name="factor_prest_co">'Supuestos'!$C$21</definedName>
-    <definedName name="jornada_semanal_co">'Supuestos'!$C$22</definedName>
-    <definedName name="horas_lab_mes_co">'Supuestos'!$C$23</definedName>
-    <definedName name="pct_nocturno">'Supuestos'!$C$24</definedName>
-    <definedName name="recargo_noct_co">'Supuestos'!$C$25</definedName>
-    <definedName name="trm_cop_usd">'Supuestos'!$C$26</definedName>
-    <definedName name="costo_hora_co">'Supuestos'!$C$27</definedName>
-    <definedName name="salario_es_eur">'Supuestos'!$C$29</definedName>
-    <definedName name="ss_empresa_es">'Supuestos'!$C$30</definedName>
-    <definedName name="horas_anuales_es">'Supuestos'!$C$31</definedName>
-    <definedName name="plus_noct_es">'Supuestos'!$C$32</definedName>
-    <definedName name="usd_por_eur">'Supuestos'!$C$33</definedName>
-    <definedName name="costo_hora_es">'Supuestos'!$C$34</definedName>
-    <definedName name="muestreo_act">'Supuestos'!$C$36</definedName>
-    <definedName name="pct_subidas">'Supuestos'!$C$37</definedName>
-    <definedName name="kb_imagen">'Supuestos'!$C$38</definedName>
-    <definedName name="img_dia_estacion">'Supuestos'!$C$39</definedName>
-    <definedName name="gb_imagenes_mes_est">'Supuestos'!$C$40</definedName>
-    <definedName name="dias_hot">'Supuestos'!$C$41</definedName>
-    <definedName name="dias_cool">'Supuestos'!$C$42</definedName>
-    <definedName name="dias_archivo">'Supuestos'!$C$43</definedName>
-    <definedName name="gb_auditoria">'Supuestos'!$C$44</definedName>
-    <definedName name="msgs_telemetria_dia">'Supuestos'!$C$45</definedName>
-    <definedName name="msgs_dia_estacion">'Supuestos'!$C$46</definedName>
-    <definedName name="gb_logs_mes">'Supuestos'!$C$47</definedName>
-    <definedName name="conv_dia_base">'Supuestos'!$C$49</definedName>
-    <definedName name="conv_dia_estacion">'Supuestos'!$C$50</definedName>
-    <definedName name="conv_mes">'Supuestos'!$C$51</definedName>
-    <definedName name="tok_in_conv">'Supuestos'!$C$52</definedName>
-    <definedName name="tok_out_conv">'Supuestos'!$C$53</definedName>
-    <definedName name="pct_cache">'Supuestos'!$C$54</definedName>
-    <definedName name="pct_modelo_grande">'Supuestos'!$C$55</definedName>
-    <definedName name="tok_embed_mes">'Supuestos'!$C$56</definedName>
-    <definedName name="capex_pc">'Supuestos'!$C$58</definedName>
-    <definedName name="capex_camara">'Supuestos'!$C$59</definedName>
-    <definedName name="capex_integracion">'Supuestos'!$C$60</definedName>
-    <definedName name="capex_planta">'Supuestos'!$C$61</definedName>
-    <definedName name="pct_mant_hw">'Supuestos'!$C$62</definedName>
-    <definedName name="replicas_agente">'Supuestos'!$C$64</definedName>
-    <definedName name="replicas_bd">'Supuestos'!$C$65</definedName>
-    <definedName name="horas_activas_vision_cloud">'Supuestos'!$C$66</definedName>
-    <definedName name="horas_entrenamiento">'Supuestos'!$C$67</definedName>
-    <definedName name="uplift_ue">'Supuestos'!$C$68</definedName>
+    <definedName name="pct_automatizado_pesimista">'Supuestos'!$C$17</definedName>
+    <definedName name="min_caso_revision">'Supuestos'!$C$18</definedName>
+    <definedName name="fraccion_atencion">'Supuestos'!$C$19</definedName>
+    <definedName name="salario_co_cop">'Supuestos'!$C$21</definedName>
+    <definedName name="factor_prest_co">'Supuestos'!$C$22</definedName>
+    <definedName name="jornada_semanal_co">'Supuestos'!$C$23</definedName>
+    <definedName name="horas_lab_mes_co">'Supuestos'!$C$24</definedName>
+    <definedName name="pct_nocturno">'Supuestos'!$C$25</definedName>
+    <definedName name="recargo_noct_co">'Supuestos'!$C$26</definedName>
+    <definedName name="trm_cop_usd">'Supuestos'!$C$27</definedName>
+    <definedName name="costo_hora_co">'Supuestos'!$C$28</definedName>
+    <definedName name="salario_es_eur">'Supuestos'!$C$30</definedName>
+    <definedName name="ss_empresa_es">'Supuestos'!$C$31</definedName>
+    <definedName name="horas_anuales_es">'Supuestos'!$C$32</definedName>
+    <definedName name="plus_noct_es">'Supuestos'!$C$33</definedName>
+    <definedName name="usd_por_eur">'Supuestos'!$C$34</definedName>
+    <definedName name="costo_hora_es">'Supuestos'!$C$35</definedName>
+    <definedName name="muestreo_act">'Supuestos'!$C$37</definedName>
+    <definedName name="pct_subidas">'Supuestos'!$C$38</definedName>
+    <definedName name="kb_imagen">'Supuestos'!$C$39</definedName>
+    <definedName name="img_dia_estacion">'Supuestos'!$C$40</definedName>
+    <definedName name="gb_imagenes_mes_est">'Supuestos'!$C$41</definedName>
+    <definedName name="dias_hot">'Supuestos'!$C$42</definedName>
+    <definedName name="dias_cool">'Supuestos'!$C$43</definedName>
+    <definedName name="dias_archivo">'Supuestos'!$C$44</definedName>
+    <definedName name="gb_auditoria">'Supuestos'!$C$45</definedName>
+    <definedName name="msgs_telemetria_dia">'Supuestos'!$C$46</definedName>
+    <definedName name="msgs_dia_estacion">'Supuestos'!$C$47</definedName>
+    <definedName name="gb_logs_mes">'Supuestos'!$C$48</definedName>
+    <definedName name="conv_dia_base">'Supuestos'!$C$50</definedName>
+    <definedName name="conv_dia_estacion">'Supuestos'!$C$51</definedName>
+    <definedName name="conv_mes">'Supuestos'!$C$52</definedName>
+    <definedName name="tok_in_conv">'Supuestos'!$C$53</definedName>
+    <definedName name="tok_out_conv">'Supuestos'!$C$54</definedName>
+    <definedName name="pct_cache">'Supuestos'!$C$55</definedName>
+    <definedName name="pct_modelo_grande">'Supuestos'!$C$56</definedName>
+    <definedName name="tok_embed_mes">'Supuestos'!$C$57</definedName>
+    <definedName name="capex_pc">'Supuestos'!$C$59</definedName>
+    <definedName name="capex_camara">'Supuestos'!$C$60</definedName>
+    <definedName name="capex_integracion">'Supuestos'!$C$61</definedName>
+    <definedName name="capex_planta">'Supuestos'!$C$62</definedName>
+    <definedName name="pct_mant_hw">'Supuestos'!$C$63</definedName>
+    <definedName name="replicas_agente">'Supuestos'!$C$65</definedName>
+    <definedName name="replicas_bd">'Supuestos'!$C$66</definedName>
+    <definedName name="horas_activas_vision_cloud">'Supuestos'!$C$67</definedName>
+    <definedName name="horas_entrenamiento">'Supuestos'!$C$68</definedName>
+    <definedName name="uplift_ue">'Supuestos'!$C$69</definedName>
     <definedName name="actual_mes_co">'Operación actual'!$B$10</definedName>
     <definedName name="actual_mes_es">'Operación actual'!$C$10</definedName>
     <definedName name="actual_estacion_co">'Operación actual'!$B$8</definedName>
@@ -151,7 +152,7 @@
       <color rgb="001F4E9E"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -183,6 +184,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -210,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -248,6 +254,8 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -644,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1095,30 +1103,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>min_caso_revision</t>
+          <t>pct_automatizado_pesimista</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Minutos humanos por caso en cola (REVIEW/REJECT)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="n">
-        <v>0.5</v>
+          <t>% automatizado en el escenario pesimista (objetos desconocidos mezclados)</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.737</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>min/caso</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Supuesto</t>
+          <t>Medido</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Mirar evidencia + reubicar el objeto desviado (~30 s)</t>
+          <t>vision-1.0.1, variante D (desconocidos mezclados): 73,7-74,9%. Se usa el extremo bajo</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1130,103 +1138,103 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>min_caso_revision</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Minutos humanos por caso en cola (REVIEW/REJECT)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>min/caso</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Mirar evidencia + reubicar el objeto desviado (~30 s)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>fraccion_atencion</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Fracción de las horas de operación de la estación que requiere una persona (supervisión itinerante, atascos, reabastecer)</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C19" s="10" t="n">
         <v>0.1</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>% horas puesto</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Horas residuales = fracción × horas_mes × factor_cobertura (≈ 60 h pagadas/mes). NO es FTE</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Costo laboral — escenario Colombia</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>salario_co_cop</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Salario base mensual operador</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>1750000</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>COP/mes</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>≈1,2 SMMLV 2025 (1.423.500 COP, Decreto 1572/2024). Actualizar con SMMLV 2026</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>factor_prest_co</t>
+          <t>salario_co_cop</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Factor prestacional (prestaciones, seguridad social, parafiscales, aux. transporte)</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="n">
-        <v>1.55</v>
+          <t>Salario base mensual operador</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>1750000</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>COP/mes</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1236,7 +1244,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Rango típico 1,50-1,60</t>
+          <t>≈1,2 SMMLV 2025 (1.423.500 COP, Decreto 1572/2024). Actualizar con SMMLV 2026</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1248,30 +1256,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>jornada_semanal_co</t>
+          <t>factor_prest_co</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Jornada máxima semanal</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>42</v>
+          <t>Factor prestacional (prestaciones, seguridad social, parafiscales, aux. transporte)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>1.55</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>h/semana</t>
+          <t>×</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Referencia</t>
+          <t>Supuesto</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Ley 2101 de 2021: 42 h/semana desde el 15-jul-2026 (Circular MinTrabajo 0101 de 2025)</t>
+          <t>Rango típico 1,50-1,60</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1283,31 +1291,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>horas_lab_mes_co</t>
+          <t>jornada_semanal_co</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Horas laborales contratadas por mes</t>
-        </is>
-      </c>
-      <c r="C23" s="8">
-        <f>jornada_semanal_co*semanas_mes</f>
-        <v/>
+          <t>Jornada máxima semanal</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>42</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>h/mes</t>
+          <t>h/semana</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Calculado</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>42 × 4,33 ≈ 182 h</t>
+          <t>Ley 2101 de 2021: 42 h/semana desde el 15-jul-2026 (Circular MinTrabajo 0101 de 2025)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1319,30 +1326,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>pct_nocturno</t>
+          <t>horas_lab_mes_co</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>% de horas en franja nocturna</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="n">
-        <v>0.33</v>
+          <t>Horas laborales contratadas por mes</t>
+        </is>
+      </c>
+      <c r="C24" s="8">
+        <f>jornada_semanal_co*semanas_mes</f>
+        <v/>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>h/mes</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Supuesto</t>
+          <t>Calculado</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>1 de 3 turnos nocturno</t>
+          <t>42 × 4,33 ≈ 182 h</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1354,16 +1362,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>recargo_noct_co</t>
+          <t>pct_nocturno</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Recargo nocturno</t>
+          <t>% de horas en franja nocturna</t>
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1372,12 +1380,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Referencia</t>
+          <t>Supuesto</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Código Sustantivo del Trabajo art. 168</t>
+          <t>1 de 3 turnos nocturno</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1389,30 +1397,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>trm_cop_usd</t>
+          <t>recargo_noct_co</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Tasa de cambio COP por USD</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>4000</v>
+          <t>Recargo nocturno</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>0.35</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>COP/USD</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Supuesto</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Verificar TRM del día (banrep.gov.co)</t>
+          <t>Código Sustantivo del Trabajo art. 168</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1424,100 +1432,100 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>trm_cop_usd</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Tasa de cambio COP por USD</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>COP/USD</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Verificar TRM del día (banrep.gov.co)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>costo_hora_co</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Costo cargado por hora-persona (Colombia)</t>
         </is>
       </c>
-      <c r="C27" s="11">
+      <c r="C28" s="11">
         <f>salario_co_cop*factor_prest_co/horas_lab_mes_co/trm_cop_usd*(1+recargo_noct_co*pct_nocturno)</f>
         <v/>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>USD/h</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Costo laboral — escenario España</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>salario_es_eur</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Salario bruto anual operador</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>22000</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>EUR/año</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Rango de convenios de industria/logística</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ss_empresa_es</t>
+          <t>salario_es_eur</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Seguridad Social a cargo de la empresa</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>0.32</v>
+          <t>Salario bruto anual operador</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>22000</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>EUR/año</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1527,7 +1535,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>≈31-33%</t>
+          <t>Rango de convenios de industria/logística</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1539,20 +1547,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>horas_anuales_es</t>
+          <t>ss_empresa_es</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Horas efectivas anuales por convenio</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>1760</v>
+          <t>Seguridad Social a cargo de la empresa</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>0.32</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>h/año</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1562,7 +1570,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Rango 1.750-1.800 h</t>
+          <t>≈31-33%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1574,20 +1582,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>plus_noct_es</t>
+          <t>horas_anuales_es</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Plus de nocturnidad</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="n">
-        <v>0.25</v>
+          <t>Horas efectivas anuales por convenio</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>1760</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>h/año</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1597,7 +1605,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>ET art. 36 remite a convenio; 25% habitual</t>
+          <t>Rango 1.750-1.800 h</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1609,20 +1617,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>usd_por_eur</t>
+          <t>plus_noct_es</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>USD por EUR</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="n">
-        <v>1.15</v>
+          <t>Plus de nocturnidad</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>0.25</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>USD/EUR</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1632,7 +1640,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Verificar tipo de cambio del día (BCE)</t>
+          <t>ET art. 36 remite a convenio; 25% habitual</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1644,97 +1652,96 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>usd_por_eur</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>USD por EUR</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>USD/EUR</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Verificar tipo de cambio del día (BCE)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>costo_hora_es</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Costo cargado por hora-persona (España)</t>
         </is>
       </c>
-      <c r="C34" s="11">
+      <c r="C35" s="11">
         <f>salario_es_eur*(1+ss_empresa_es)/horas_anuales_es*usd_por_eur*(1+plus_noct_es*pct_nocturno)</f>
         <v/>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>USD/h</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Imágenes y telemetría</t>
         </is>
       </c>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>muestreo_act</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>% de imágenes ACT que se suben a la nube</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Todas las REVIEW/REJECT + muestra de ACT</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>pct_subidas</t>
+          <t>muestreo_act</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>% de imágenes subidas a la nube</t>
-        </is>
-      </c>
-      <c r="C37" s="12">
-        <f>(1-pct_automatizado)+pct_automatizado*muestreo_act</f>
-        <v/>
+          <t>% de imágenes ACT que se suben a la nube</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>0.02</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1743,10 +1750,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Calculado</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr"/>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Todas las REVIEW/REJECT + muestra de ACT</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -1756,32 +1767,29 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>kb_imagen</t>
+          <t>pct_subidas</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Tamaño medio por imagen subida (JPEG, anonimizada)</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>150</v>
+          <t>% de imágenes subidas a la nube</t>
+        </is>
+      </c>
+      <c r="C38" s="12">
+        <f>(1-pct_automatizado)+pct_automatizado*muestreo_act</f>
+        <v/>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Cámara ~1,3 MP comprimida</t>
-        </is>
-      </c>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -1791,31 +1799,30 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>img_dia_estacion</t>
+          <t>kb_imagen</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Imágenes subidas por día por estación</t>
-        </is>
-      </c>
-      <c r="C39" s="13">
-        <f>throughput_obj_h*24*pct_subidas</f>
-        <v/>
+          <t>Tamaño medio por imagen subida (JPEG, anonimizada)</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>150</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>img/día</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Calculado</t>
+          <t>Supuesto</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Se suben directo a Blob/S3 desde el borde (no por IoT Hub/IoT Core)</t>
+          <t>Cámara ~1,3 MP comprimida</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1827,21 +1834,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>gb_imagenes_mes_est</t>
+          <t>img_dia_estacion</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>GB de imágenes nuevas por mes por estación</t>
-        </is>
-      </c>
-      <c r="C40" s="8">
-        <f>throughput_obj_h*horas_mes*pct_subidas*kb_imagen/1024/1024</f>
+          <t>Imágenes subidas por día por estación</t>
+        </is>
+      </c>
+      <c r="C40" s="13">
+        <f>throughput_obj_h*24*pct_subidas</f>
         <v/>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>GB/mes</t>
+          <t>img/día</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1849,7 +1856,11 @@
           <t>Calculado</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Se suben directo a Blob/S3 desde el borde (no por IoT Hub/IoT Core)</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -1859,25 +1870,26 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dias_hot</t>
+          <t>gb_imagenes_mes_est</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Días en tier caliente (Hot / S3 Standard)</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="n">
-        <v>30</v>
+          <t>GB de imágenes nuevas por mes por estación</t>
+        </is>
+      </c>
+      <c r="C41" s="8">
+        <f>throughput_obj_h*horas_mes*pct_subidas*kb_imagen/1024/1024</f>
+        <v/>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>días</t>
+          <t>GB/mes</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Supuesto</t>
+          <t>Calculado</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
@@ -1890,16 +1902,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>dias_cool</t>
+          <t>dias_hot</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Días en tier frío (Cool / S3 Standard-IA)</t>
+          <t>Días en tier caliente (Hot / S3 Standard)</t>
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1911,11 +1923,7 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>Del día 31 al 180</t>
-        </is>
-      </c>
+      <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -1925,16 +1933,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>dias_archivo</t>
+          <t>dias_cool</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Días en archivo (Archive / Glacier Deep Archive)</t>
+          <t>Días en tier frío (Cool / S3 Standard-IA)</t>
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>915</v>
+        <v>150</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1948,7 +1956,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Hasta 3 años de retención</t>
+          <t>Del día 31 al 180</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1960,20 +1968,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>gb_auditoria</t>
+          <t>dias_archivo</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>GB acumulados en la cuenta de auditoría (ZRS, inmutable)</t>
+          <t>Días en archivo (Archive / Glacier Deep Archive)</t>
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>20</v>
+        <v>915</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>días</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1983,7 +1991,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Exportación diaria de la tabla de auditoría</t>
+          <t>Hasta 3 años de retención</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1995,20 +2003,20 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>msgs_telemetria_dia</t>
+          <t>gb_auditoria</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Mensajes de telemetría por día por estación (≤ 4 KB)</t>
+          <t>GB acumulados en la cuenta de auditoría (ZRS, inmutable)</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>3000</v>
+        <v>20</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>msgs/día</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2018,7 +2026,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Métricas agregadas cada 30 s + eventos</t>
+          <t>Exportación diaria de la tabla de auditoría</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2030,17 +2038,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>msgs_dia_estacion</t>
+          <t>msgs_telemetria_dia</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Mensajes IoT por día por estación (telemetría + 1 aviso de metadatos por imagen subida)</t>
-        </is>
-      </c>
-      <c r="C46" s="13">
-        <f>msgs_telemetria_dia+img_dia_estacion</f>
-        <v/>
+          <t>Mensajes de telemetría por día por estación (≤ 4 KB)</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>3000</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2049,12 +2056,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Calculado</t>
+          <t>Supuesto</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Los bytes de la imagen no pasan por IoT Hub; solo un mensaje pequeño con su referencia</t>
+          <t>Métricas agregadas cada 30 s + eventos</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2066,95 +2073,100 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>msgs_dia_estacion</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Mensajes IoT por día por estación (telemetría + 1 aviso de metadatos por imagen subida)</t>
+        </is>
+      </c>
+      <c r="C47" s="13">
+        <f>msgs_telemetria_dia+img_dia_estacion</f>
+        <v/>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>msgs/día</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Los bytes de la imagen no pasan por IoT Hub; solo un mensaje pequeño con su referencia</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>gb_logs_mes</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>GB de logs / trazas por mes</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n">
+      <c r="C48" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>GB/mes</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F48" s="3" t="inlineStr">
         <is>
           <t>Con muestreo de trazas</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Asistente agéntico (LLM)</t>
         </is>
       </c>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>conv_dia_base</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Conversaciones por día (base por planta)</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>conv/día</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>conv_dia_estacion</t>
+          <t>conv_dia_base</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Conversaciones adicionales por día por estación</t>
+          <t>Conversaciones por día (base por planta)</t>
         </is>
       </c>
       <c r="C50" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2176,26 +2188,25 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>conv_mes</t>
+          <t>conv_dia_estacion</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Conversaciones por mes</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>(conv_dia_base+conv_dia_estacion*estaciones)*dias_mes</f>
-        <v/>
+          <t>Conversaciones adicionales por día por estación</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>20</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>conv/mes</t>
+          <t>conv/día</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Calculado</t>
+          <t>Supuesto</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr"/>
@@ -2208,32 +2219,29 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>tok_in_conv</t>
+          <t>conv_mes</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Tokens de entrada por conversación (multi-turno, con tools)</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="n">
-        <v>25000</v>
+          <t>Conversaciones por mes</t>
+        </is>
+      </c>
+      <c r="C52" s="13">
+        <f>(conv_dia_base+conv_dia_estacion*estaciones)*dias_mes</f>
+        <v/>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>conv/mes</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>Medir con `usage` del agente</t>
-        </is>
-      </c>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2243,16 +2251,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>tok_out_conv</t>
+          <t>tok_in_conv</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Tokens de salida por conversación</t>
+          <t>Tokens de entrada por conversación (multi-turno, con tools)</t>
         </is>
       </c>
       <c r="C53" s="7" t="n">
-        <v>1500</v>
+        <v>25000</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2264,7 +2272,11 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Medir con `usage` del agente</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2274,20 +2286,20 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>pct_cache</t>
+          <t>tok_out_conv</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>% de tokens de entrada servidos desde caché</t>
-        </is>
-      </c>
-      <c r="C54" s="10" t="n">
-        <v>0.5</v>
+          <t>Tokens de salida por conversación</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>1500</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>tokens</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2295,11 +2307,7 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>Prompt de sistema y tools estables</t>
-        </is>
-      </c>
+      <c r="F54" s="3" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2309,16 +2317,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>pct_modelo_grande</t>
+          <t>pct_cache</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>% de conversaciones enrutadas al modelo grande</t>
+          <t>% de tokens de entrada servidos desde caché</t>
         </is>
       </c>
       <c r="C55" s="10" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2332,7 +2340,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Solo diagnósticos complejos</t>
+          <t>Prompt de sistema y tools estables</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2344,95 +2352,95 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>pct_modelo_grande</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>% de conversaciones enrutadas al modelo grande</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Solo diagnósticos complejos</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>tok_embed_mes</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Tokens de embeddings por mes (reindexado SOP)</t>
         </is>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C57" s="7" t="n">
         <v>2000000</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>tokens</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr"/>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>CAPEX e implementación (pago único)</t>
         </is>
       </c>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="6" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>capex_pc</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>PC industrial fanless por estación</t>
-        </is>
-      </c>
-      <c r="C58" s="14" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Rango de mercado USD 2.000-4.000</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="6" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>capex_camara</t>
+          <t>capex_pc</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Cámara industrial + óptica + iluminación + soporte</t>
+          <t>PC industrial fanless por estación</t>
         </is>
       </c>
       <c r="C59" s="14" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2444,7 +2452,11 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Rango de mercado USD 2.000-4.000</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2454,16 +2466,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>capex_integracion</t>
+          <t>capex_camara</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Integración PLC/robot y puesta en marcha por estación</t>
+          <t>Cámara industrial + óptica + iluminación + soporte</t>
         </is>
       </c>
       <c r="C60" s="14" t="n">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2475,11 +2487,7 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>Ingeniería de automatización, calibración, FAT/SAT</t>
-        </is>
-      </c>
+      <c r="F60" s="3" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2489,16 +2497,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>capex_planta</t>
+          <t>capex_integracion</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Implementación por planta (piloto, validación, capacitación, nube)</t>
+          <t>Integración PLC/robot y puesta en marcha por estación</t>
         </is>
       </c>
       <c r="C61" s="14" t="n">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2510,7 +2518,11 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniería de automatización, calibración, FAT/SAT</t>
+        </is>
+      </c>
       <c r="G61" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2520,20 +2532,20 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>pct_mant_hw</t>
+          <t>capex_planta</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Mantenimiento anual del hardware de borde</t>
-        </is>
-      </c>
-      <c r="C62" s="10" t="n">
-        <v>0.1</v>
+          <t>Implementación por planta (piloto, validación, capacitación, nube)</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="n">
+        <v>30000</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>%/año</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2549,62 +2561,58 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>pct_mant_hw</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Mantenimiento anual del hardware de borde</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>%/año</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>Producción en la nube</t>
         </is>
       </c>
-      <c r="B63" s="6" t="n"/>
-      <c r="C63" s="6" t="n"/>
-      <c r="D63" s="6" t="n"/>
-      <c r="E63" s="6" t="n"/>
-      <c r="F63" s="6" t="n"/>
-      <c r="G63" s="6" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>replicas_agente</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Réplicas mínimas del agente en horario de turnos</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>réplicas</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Supuesto</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>≥ 2 para que la redundancia de zona de Container Apps / ECS en 2 AZ sea real</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>replicas_bd</t>
+          <t>replicas_agente</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Réplicas de base de datos (1 = sin HA, 2 = HA de zona)</t>
+          <t>Réplicas mínimas del agente en horario de turnos</t>
         </is>
       </c>
       <c r="C65" s="7" t="n">
@@ -2622,7 +2630,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Producción: HA. Piloto: 1</t>
+          <t>≥ 2 para que la redundancia de zona de Container Apps / ECS en 2 AZ sea real</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2634,20 +2642,20 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>horas_activas_vision_cloud</t>
+          <t>replicas_bd</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Horas activas/mes del servicio de visión en nube (no tiempo real)</t>
+          <t>Réplicas de base de datos (1 = sin HA, 2 = HA de zona)</t>
         </is>
       </c>
       <c r="C66" s="7" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>h/mes</t>
+          <t>réplicas</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2657,7 +2665,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Escala a cero</t>
+          <t>Producción: HA. Piloto: 1</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2669,16 +2677,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>horas_entrenamiento</t>
+          <t>horas_activas_vision_cloud</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Horas de cómputo de reentrenamiento al mes</t>
+          <t>Horas activas/mes del servicio de visión en nube (no tiempo real)</t>
         </is>
       </c>
       <c r="C67" s="7" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2690,7 +2698,11 @@
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F67" s="3" t="inlineStr"/>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Escala a cero</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -2700,33 +2712,64 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>horas_entrenamiento</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Horas de cómputo de reentrenamiento al mes</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>h/mes</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Supuesto</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>uplift_ue</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>Factor de precio UE vs EE. UU. cuando no hay precio UE verificado</t>
         </is>
       </c>
-      <c r="C68" s="9" t="n">
+      <c r="C69" s="9" t="n">
         <v>1.1</v>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>×</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>Supuesto</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>Solo se usa en filas UE marcadas 'Estimado (US × factor UE)'</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
@@ -8057,7 +8100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -8070,7 +8113,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Comparativo: operación actual vs Azure vs AWS</t>
+          <t>Comparativo: operación actual vs Azure vs AWS (base = pct_automatizado; abajo, escenario pesimista)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -8541,36 +8584,89 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>ESCENARIO PESIMISTA (pct_automatizado_pesimista, desconocidos mezclados)</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Lectura rápida:</t>
-        </is>
+          <t>Ahorro mensual pesimista</t>
+        </is>
+      </c>
+      <c r="B26" s="31">
+        <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-pct_automatizado_pesimista)+pct_automatizado_pesimista*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-pct_automatizado_pesimista)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="C26" s="31">
+        <f>actual_mes_co-((aws_total_mes-aws_img_mes+aws_img_mes*((1-pct_automatizado_pesimista)+pct_automatizado_pesimista*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-pct_automatizado_pesimista)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31">
+        <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-pct_automatizado_pesimista)+pct_automatizado_pesimista*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-pct_automatizado_pesimista)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
+      </c>
+      <c r="E26" s="31">
+        <f>actual_mes_es-((aws_total_mes_ue-aws_img_mes_ue+aws_img_mes_ue*((1-pct_automatizado_pesimista)+pct_automatizado_pesimista*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-pct_automatizado_pesimista)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• El ahorro viene de retirar 3 turnos de operador por estación; la nube es una fracción pequeña del costo laboral evitado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>• El factor que más mueve el resultado es % automatizado (cola de revisión) y el costo laboral local, no el proveedor de nube.</t>
-        </is>
+          <t>Payback pesimista (meses)</t>
+        </is>
+      </c>
+      <c r="B27" s="32">
+        <f>IF(B26&gt;0,B17/B26,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="C27" s="32">
+        <f>IF(C26&gt;0,C17/C26,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="D27" s="32">
+        <f>IF(D26&gt;0,D17/D26,"No recupera")</f>
+        <v/>
+      </c>
+      <c r="E27" s="32">
+        <f>IF(E26&gt;0,E17/E26,"No recupera")</f>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• Con 1 estación en Colombia el payback es largo: el CAPEX de implementación por planta pesa mucho (ver Sensibilidad).</t>
+          <t>Lectura rápida:</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
+        <is>
+          <t>• El ahorro viene de retirar 3 turnos de operador por estación; la nube es una fracción pequeña del costo laboral evitado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>• El factor que más mueve el resultado es % automatizado (cola de revisión) y el costo laboral local, no el proveedor de nube.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>• Con 1 estación en Colombia el payback es largo: el CAPEX de implementación por planta pesa mucho (ver Sensibilidad).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>• Ningún número de esta hoja está hardcodeado: todo sale de Supuestos, Operación actual, Azure y AWS.</t>
         </is>
@@ -8667,204 +8763,204 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31" t="n">
+      <c r="A6" s="33" t="n">
         <v>0.737</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A6)+$A6*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D6" s="33">
+      <c r="D6" s="35">
         <f>IF(C6&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C6,"No recupera")</f>
         <v/>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A6)+$A6*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A6)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G6" s="33">
+      <c r="G6" s="35">
         <f>IF(F6&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F6,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="n">
+      <c r="A7" s="33" t="n">
         <v>0.749</v>
       </c>
-      <c r="B7" s="32">
+      <c r="B7" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A7)+$A7*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="35">
         <f>IF(C7&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C7,"No recupera")</f>
         <v/>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A7)+$A7*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A7)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G7" s="33">
+      <c r="G7" s="35">
         <f>IF(F7&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F7,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="31" t="n">
+      <c r="A8" s="33" t="n">
         <v>0.8</v>
       </c>
-      <c r="B8" s="32">
+      <c r="B8" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A8)+$A8*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D8" s="33">
+      <c r="D8" s="35">
         <f>IF(C8&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C8,"No recupera")</f>
         <v/>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A8)+$A8*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A8)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G8" s="33">
+      <c r="G8" s="35">
         <f>IF(F8&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F8,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="n">
+      <c r="A9" s="33" t="n">
         <v>0.9</v>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C9" s="32">
+      <c r="C9" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A9)+$A9*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D9" s="33">
+      <c r="D9" s="35">
         <f>IF(C9&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C9,"No recupera")</f>
         <v/>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A9)+$A9*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A9)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G9" s="33">
+      <c r="G9" s="35">
         <f>IF(F9&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F9,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="n">
+      <c r="A10" s="33" t="n">
         <v>0.903</v>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A10)+$A10*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="35">
         <f>IF(C10&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C10,"No recupera")</f>
         <v/>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A10)+$A10*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A10)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="35">
         <f>IF(F10&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F10,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="n">
+      <c r="A11" s="33" t="n">
         <v>0.95</v>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A11)+$A11*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="35">
         <f>IF(C11&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C11,"No recupera")</f>
         <v/>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A11)+$A11*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A11)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G11" s="33">
+      <c r="G11" s="35">
         <f>IF(F11&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F11,"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="n">
+      <c r="A12" s="33" t="n">
         <v>0.99</v>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_co</f>
         <v/>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="34">
         <f>actual_mes_co-((azure_total_mes-azure_img_mes+azure_img_mes*((1-$A12)+$A12*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_co+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co)</f>
         <v/>
       </c>
-      <c r="D12" s="33">
+      <c r="D12" s="35">
         <f>IF(C12&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/C12,"No recupera")</f>
         <v/>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="34">
         <f>estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_es</f>
         <v/>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="34">
         <f>actual_mes_es-((azure_total_mes_ue-azure_img_mes_ue+azure_img_mes_ue*((1-$A12)+$A12*muestreo_act)/pct_subidas)*plantas+estaciones*plantas*(capex_pc+capex_camara)*pct_mant_hw/12+estaciones*plantas*throughput_obj_h*horas_mes*(1-$A12)*min_caso_revision/60*costo_hora_es+estaciones*plantas*fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es)</f>
         <v/>
       </c>
-      <c r="G12" s="33">
+      <c r="G12" s="35">
         <f>IF(F12&gt;0,(estaciones*plantas*(capex_pc+capex_camara+capex_integracion)+capex_planta*plantas)/F12,"No recupera")</f>
         <v/>
       </c>
@@ -8929,88 +9025,88 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="34" t="n">
+      <c r="A17" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="34">
         <f>actual_estacion_co*$A17*plantas</f>
         <v/>
       </c>
-      <c r="C17" s="32">
+      <c r="C17" s="34">
         <f>(azure_fijo_mes+azure_por_estacion_mes*$A17+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A17)*dias_mes)*plantas+$A17*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
         <v/>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="35">
         <f>IF(B17&gt;C17,($A17*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B17-C17),"No recupera")</f>
         <v/>
       </c>
-      <c r="E17" s="32">
+      <c r="E17" s="34">
         <f>actual_estacion_es*$A17*plantas</f>
         <v/>
       </c>
-      <c r="F17" s="32">
+      <c r="F17" s="34">
         <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A17+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A17)*dias_mes)*plantas+$A17*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
         <v/>
       </c>
-      <c r="G17" s="33">
+      <c r="G17" s="35">
         <f>IF(E17&gt;F17,($A17*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E17-F17),"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="34" t="n">
+      <c r="A18" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="B18" s="32">
+      <c r="B18" s="34">
         <f>actual_estacion_co*$A18*plantas</f>
         <v/>
       </c>
-      <c r="C18" s="32">
+      <c r="C18" s="34">
         <f>(azure_fijo_mes+azure_por_estacion_mes*$A18+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A18)*dias_mes)*plantas+$A18*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
         <v/>
       </c>
-      <c r="D18" s="33">
+      <c r="D18" s="35">
         <f>IF(B18&gt;C18,($A18*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B18-C18),"No recupera")</f>
         <v/>
       </c>
-      <c r="E18" s="32">
+      <c r="E18" s="34">
         <f>actual_estacion_es*$A18*plantas</f>
         <v/>
       </c>
-      <c r="F18" s="32">
+      <c r="F18" s="34">
         <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A18+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A18)*dias_mes)*plantas+$A18*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
         <v/>
       </c>
-      <c r="G18" s="33">
+      <c r="G18" s="35">
         <f>IF(E18&gt;F18,($A18*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E18-F18),"No recupera")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="n">
+      <c r="A19" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="34">
         <f>actual_estacion_co*$A19*plantas</f>
         <v/>
       </c>
-      <c r="C19" s="32">
+      <c r="C19" s="34">
         <f>(azure_fijo_mes+azure_por_estacion_mes*$A19+azure_llm_por_conv*(conv_dia_base+conv_dia_estacion*$A19)*dias_mes)*plantas+$A19*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_co+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_co+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
         <v/>
       </c>
-      <c r="D19" s="33">
+      <c r="D19" s="35">
         <f>IF(B19&gt;C19,($A19*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(B19-C19),"No recupera")</f>
         <v/>
       </c>
-      <c r="E19" s="32">
+      <c r="E19" s="34">
         <f>actual_estacion_es*$A19*plantas</f>
         <v/>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="34">
         <f>(azure_fijo_mes_ue+azure_por_estacion_mes_ue*$A19+azure_llm_por_conv_ue*(conv_dia_base+conv_dia_estacion*$A19)*dias_mes)*plantas+$A19*plantas*(throughput_obj_h*horas_mes*(1-pct_automatizado)*min_caso_revision/60*costo_hora_es+fraccion_atencion*horas_mes*factor_cobertura*costo_hora_es+(capex_pc+capex_camara)*pct_mant_hw/12)</f>
         <v/>
       </c>
-      <c r="G19" s="33">
+      <c r="G19" s="35">
         <f>IF(E19&gt;F19,($A19*(capex_pc+capex_camara+capex_integracion)+capex_planta)*plantas/(E19-F19),"No recupera")</f>
         <v/>
       </c>
@@ -9052,18 +9148,18 @@
       <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="34" t="n">
+      <c r="A24" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="34">
         <f>azure_llm_por_conv*$A24*dias_mes</f>
         <v/>
       </c>
-      <c r="C24" s="32">
+      <c r="C24" s="34">
         <f>aws_llm_por_conv*$A24*dias_mes</f>
         <v/>
       </c>
-      <c r="D24" s="32">
+      <c r="D24" s="34">
         <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A24*dias_mes</f>
         <v/>
       </c>
@@ -9073,18 +9169,18 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="34" t="n">
+      <c r="A25" s="36" t="n">
         <v>60</v>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="34">
         <f>azure_llm_por_conv*$A25*dias_mes</f>
         <v/>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="34">
         <f>aws_llm_por_conv*$A25*dias_mes</f>
         <v/>
       </c>
-      <c r="D25" s="32">
+      <c r="D25" s="34">
         <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A25*dias_mes</f>
         <v/>
       </c>
@@ -9094,18 +9190,18 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="34" t="n">
+      <c r="A26" s="36" t="n">
         <v>200</v>
       </c>
-      <c r="B26" s="32">
+      <c r="B26" s="34">
         <f>azure_llm_por_conv*$A26*dias_mes</f>
         <v/>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="34">
         <f>aws_llm_por_conv*$A26*dias_mes</f>
         <v/>
       </c>
-      <c r="D26" s="32">
+      <c r="D26" s="34">
         <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A26*dias_mes</f>
         <v/>
       </c>
@@ -9115,18 +9211,18 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="34" t="n">
+      <c r="A27" s="36" t="n">
         <v>1000</v>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="34">
         <f>azure_llm_por_conv*$A27*dias_mes</f>
         <v/>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="34">
         <f>aws_llm_por_conv*$A27*dias_mes</f>
         <v/>
       </c>
-      <c r="D27" s="32">
+      <c r="D27" s="34">
         <f>(tok_in_conv*((1-pct_cache)*azure_big_in+pct_cache*azure_big_cache)+tok_out_conv*azure_big_out)/1000*$A27*dias_mes</f>
         <v/>
       </c>
@@ -9278,7 +9374,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I5" s="35" t="inlineStr">
+      <c r="I5" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard vCPU Active Usage'</t>
         </is>
@@ -9323,7 +9419,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I6" s="35" t="inlineStr">
+      <c r="I6" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard vCPU Active Usage'</t>
         </is>
@@ -9368,7 +9464,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I7" s="35" t="inlineStr">
+      <c r="I7" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard Memory Active Usage'</t>
         </is>
@@ -9413,7 +9509,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I8" s="35" t="inlineStr">
+      <c r="I8" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Standard Memory Active Usage'</t>
         </is>
@@ -9458,7 +9554,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I9" s="35" t="inlineStr">
+      <c r="I9" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Environment Private Endpoint'</t>
         </is>
@@ -9503,7 +9599,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I10" s="35" t="inlineStr">
+      <c r="I10" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Container Apps' and meterName eq 'Environment Private Endpoint'</t>
         </is>
@@ -9548,7 +9644,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I11" s="35" t="inlineStr">
+      <c r="I11" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Container Registry' and meterName eq 'Basic Registry Unit'</t>
         </is>
@@ -9593,7 +9689,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I12" s="35" t="inlineStr">
+      <c r="I12" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Container Registry' and meterName eq 'Basic Registry Unit'</t>
         </is>
@@ -9638,7 +9734,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I13" s="35" t="inlineStr">
+      <c r="I13" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Virtual Machines' and armSkuName eq 'Standard_D4s_v3' and meterName eq 'D4s v3'</t>
         </is>
@@ -9683,7 +9779,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I14" s="35" t="inlineStr">
+      <c r="I14" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Virtual Machines' and armSkuName eq 'Standard_D4s_v3' and meterName eq 'D4s v3'</t>
         </is>
@@ -9728,7 +9824,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I15" s="35" t="inlineStr">
+      <c r="I15" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flexible Server General Purpose Ddsv5 Series Compute' and skuName eq '2 vCore'</t>
         </is>
@@ -9773,7 +9869,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I16" s="35" t="inlineStr">
+      <c r="I16" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flexible Server General Purpose Ddsv5 Series Compute' and skuName eq '2 vCore'</t>
         </is>
@@ -9818,7 +9914,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I17" s="35" t="inlineStr">
+      <c r="I17" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flex Server Storage' and meterName eq 'Storage Data Stored'</t>
         </is>
@@ -9863,7 +9959,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I18" s="35" t="inlineStr">
+      <c r="I18" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure Database for PostgreSQL Flex Server Storage' and meterName eq 'Storage Data Stored'</t>
         </is>
@@ -9908,7 +10004,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I19" s="35" t="inlineStr">
+      <c r="I19" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Azure Cognitive Search' and meterName eq 'Basic Unit'</t>
         </is>
@@ -9953,7 +10049,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I20" s="35" t="inlineStr">
+      <c r="I20" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Azure Cognitive Search' and meterName eq 'Basic Unit'</t>
         </is>
@@ -9998,7 +10094,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I21" s="35" t="inlineStr">
+      <c r="I21" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot LRS Data Stored'</t>
         </is>
@@ -10043,7 +10139,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I22" s="35" t="inlineStr">
+      <c r="I22" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot LRS Data Stored'</t>
         </is>
@@ -10088,7 +10184,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I23" s="35" t="inlineStr">
+      <c r="I23" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Cool LRS Data Stored'</t>
         </is>
@@ -10133,7 +10229,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I24" s="35" t="inlineStr">
+      <c r="I24" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Cool LRS Data Stored'</t>
         </is>
@@ -10178,7 +10274,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I25" s="35" t="inlineStr">
+      <c r="I25" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Archive LRS Data Stored'</t>
         </is>
@@ -10223,7 +10319,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I26" s="35" t="inlineStr">
+      <c r="I26" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Archive LRS Data Stored'</t>
         </is>
@@ -10268,7 +10364,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I27" s="35" t="inlineStr">
+      <c r="I27" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot ZRS Data Stored'</t>
         </is>
@@ -10313,7 +10409,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I28" s="35" t="inlineStr">
+      <c r="I28" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'General Block Blob v2' and meterName eq 'Hot ZRS Data Stored'</t>
         </is>
@@ -10358,7 +10454,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I29" s="35" t="inlineStr">
+      <c r="I29" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'IoT Hub' and meterName eq 'S1 Unit'</t>
         </is>
@@ -10403,7 +10499,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I30" s="35" t="inlineStr">
+      <c r="I30" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'westeurope' and priceType eq 'Consumption' and serviceName eq 'IoT Hub' and meterName eq 'S1 Unit'</t>
         </is>
@@ -10448,7 +10544,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I31" s="35" t="inlineStr">
+      <c r="I31" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Servers' and meterName eq 'Standard P2 Node'</t>
         </is>
@@ -10493,7 +10589,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I32" s="35" t="inlineStr">
+      <c r="I32" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Servers' and meterName eq 'Standard P2 Node'</t>
         </is>
@@ -10538,7 +10634,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I33" s="35" t="inlineStr">
+      <c r="I33" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Key Vault' and skuName eq 'Standard' and meterName eq 'Operations'</t>
         </is>
@@ -10583,7 +10679,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I34" s="35" t="inlineStr">
+      <c r="I34" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Key Vault' and skuName eq 'Standard' and meterName eq 'Operations'</t>
         </is>
@@ -10628,7 +10724,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I35" s="35" t="inlineStr">
+      <c r="I35" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and serviceName eq 'Log Analytics' and meterName eq 'Analytics Logs Data Ingestion'</t>
         </is>
@@ -10673,7 +10769,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I36" s="35" t="inlineStr">
+      <c r="I36" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and serviceName eq 'Log Analytics' and meterName eq 'Analytics Logs Data Ingestion'</t>
         </is>
@@ -10718,7 +10814,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I37" s="35" t="inlineStr">
+      <c r="I37" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Containers' and meterName eq 'Standard Images'</t>
         </is>
@@ -10763,7 +10859,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I38" s="35" t="inlineStr">
+      <c r="I38" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Microsoft Defender for Containers' and meterName eq 'Standard Images'</t>
         </is>
@@ -10808,7 +10904,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I39" s="35" t="inlineStr">
+      <c r="I39" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'text-embedding-3-small-glbl Tokens'</t>
         </is>
@@ -10853,7 +10949,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I40" s="35" t="inlineStr">
+      <c r="I40" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'text-embedding-3-small-glbl Tokens'</t>
         </is>
@@ -10898,7 +10994,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I41" s="35" t="inlineStr">
+      <c r="I41" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Inp Data Zone Tokens'</t>
         </is>
@@ -10943,7 +11039,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I42" s="35" t="inlineStr">
+      <c r="I42" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Inp Data Zone Tokens'</t>
         </is>
@@ -10988,7 +11084,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I43" s="35" t="inlineStr">
+      <c r="I43" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini cached Inp DZone Tokens'</t>
         </is>
@@ -11033,7 +11129,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I44" s="35" t="inlineStr">
+      <c r="I44" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini cached Inp DZone Tokens'</t>
         </is>
@@ -11078,7 +11174,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I45" s="35" t="inlineStr">
+      <c r="I45" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Outp Data Zone Tokens'</t>
         </is>
@@ -11123,7 +11219,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I46" s="35" t="inlineStr">
+      <c r="I46" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 mini Outp Data Zone Tokens'</t>
         </is>
@@ -11168,7 +11264,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I47" s="35" t="inlineStr">
+      <c r="I47" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Inp Data Zone Tokens'</t>
         </is>
@@ -11213,7 +11309,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I48" s="35" t="inlineStr">
+      <c r="I48" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Inp Data Zone Tokens'</t>
         </is>
@@ -11258,7 +11354,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I49" s="35" t="inlineStr">
+      <c r="I49" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 cached Inp Data Zone Tokens'</t>
         </is>
@@ -11303,7 +11399,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I50" s="35" t="inlineStr">
+      <c r="I50" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 cached Inp Data Zone Tokens'</t>
         </is>
@@ -11348,7 +11444,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I51" s="35" t="inlineStr">
+      <c r="I51" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'eastus2' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Outp Data Zone Tokens'</t>
         </is>
@@ -11393,7 +11489,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I52" s="35" t="inlineStr">
+      <c r="I52" s="37" t="inlineStr">
         <is>
           <t>https://prices.azure.com/api/retail/prices?$filter=armRegionName eq 'spaincentral' and priceType eq 'Consumption' and productName eq 'Azure OpenAI' and meterName eq 'gpt 4.1 Outp Data Zone Tokens'</t>
         </is>
@@ -11438,7 +11534,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I53" s="35" t="inlineStr">
+      <c r="I53" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/us-east-1/index.json</t>
         </is>
@@ -11483,7 +11579,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I54" s="35" t="inlineStr">
+      <c r="I54" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/eu-south-2/index.json</t>
         </is>
@@ -11528,7 +11624,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I55" s="35" t="inlineStr">
+      <c r="I55" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/us-east-1/index.json</t>
         </is>
@@ -11573,7 +11669,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I56" s="35" t="inlineStr">
+      <c r="I56" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECS/current/eu-south-2/index.json</t>
         </is>
@@ -11618,7 +11714,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I57" s="35" t="inlineStr">
+      <c r="I57" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/us-east-1/index.json</t>
         </is>
@@ -11663,7 +11759,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I58" s="35" t="inlineStr">
+      <c r="I58" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/eu-south-2/index.json</t>
         </is>
@@ -11708,7 +11804,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I59" s="35" t="inlineStr">
+      <c r="I59" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/us-east-1/index.json</t>
         </is>
@@ -11753,7 +11849,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I60" s="35" t="inlineStr">
+      <c r="I60" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSELB/current/eu-south-2/index.json</t>
         </is>
@@ -11798,7 +11894,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I61" s="35" t="inlineStr">
+      <c r="I61" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonVPC/current/us-east-1/index.json</t>
         </is>
@@ -11843,7 +11939,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I62" s="35" t="inlineStr">
+      <c r="I62" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonVPC/current/eu-south-2/index.json</t>
         </is>
@@ -11888,7 +11984,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I63" s="35" t="inlineStr">
+      <c r="I63" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECR/current/us-east-1/index.json</t>
         </is>
@@ -11933,7 +12029,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I64" s="35" t="inlineStr">
+      <c r="I64" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonECR/current/eu-south-2/index.json</t>
         </is>
@@ -11978,7 +12074,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I65" s="35" t="inlineStr">
+      <c r="I65" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonSageMaker/current/us-east-1/index.json</t>
         </is>
@@ -12023,7 +12119,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I66" s="35" t="inlineStr">
+      <c r="I66" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonSageMaker/current/eu-south-2/index.json</t>
         </is>
@@ -12068,7 +12164,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I67" s="35" t="inlineStr">
+      <c r="I67" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/us-east-1/index.json</t>
         </is>
@@ -12113,7 +12209,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I68" s="35" t="inlineStr">
+      <c r="I68" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/eu-south-2/index.json</t>
         </is>
@@ -12158,7 +12254,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I69" s="35" t="inlineStr">
+      <c r="I69" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/us-east-1/index.json</t>
         </is>
@@ -12203,7 +12299,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I70" s="35" t="inlineStr">
+      <c r="I70" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonRDS/current/eu-south-2/index.json</t>
         </is>
@@ -12248,7 +12344,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I71" s="35" t="inlineStr">
+      <c r="I71" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/us-east-1/index.json</t>
         </is>
@@ -12293,7 +12389,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I72" s="35" t="inlineStr">
+      <c r="I72" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/eu-south-2/index.json</t>
         </is>
@@ -12338,7 +12434,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I73" s="35" t="inlineStr">
+      <c r="I73" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/us-east-1/index.json</t>
         </is>
@@ -12383,7 +12479,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I74" s="35" t="inlineStr">
+      <c r="I74" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3/current/eu-south-2/index.json</t>
         </is>
@@ -12428,7 +12524,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I75" s="35" t="inlineStr">
+      <c r="I75" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3GlacierDeepArchive/current/us-east-1/index.json</t>
         </is>
@@ -12473,7 +12569,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I76" s="35" t="inlineStr">
+      <c r="I76" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonS3GlacierDeepArchive/current/eu-south-2/index.json</t>
         </is>
@@ -12518,7 +12614,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I77" s="35" t="inlineStr">
+      <c r="I77" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/us-east-1/index.json</t>
         </is>
@@ -12563,7 +12659,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I78" s="35" t="inlineStr">
+      <c r="I78" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/eu-south-2/index.json</t>
         </is>
@@ -12608,7 +12704,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I79" s="35" t="inlineStr">
+      <c r="I79" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/us-east-1/index.json</t>
         </is>
@@ -12653,7 +12749,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I80" s="35" t="inlineStr">
+      <c r="I80" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSIoT/current/eu-south-2/index.json</t>
         </is>
@@ -12698,7 +12794,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I81" s="35" t="inlineStr">
+      <c r="I81" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSGreengrass/current/us-east-1/index.json</t>
         </is>
@@ -12743,7 +12839,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I82" s="35" t="inlineStr">
+      <c r="I82" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSGreengrass/current/eu-south-2/index.json</t>
         </is>
@@ -12788,7 +12884,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I83" s="35" t="inlineStr">
+      <c r="I83" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSSecretsManager/current/us-east-1/index.json</t>
         </is>
@@ -12833,7 +12929,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I84" s="35" t="inlineStr">
+      <c r="I84" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AWSSecretsManager/current/eu-south-2/index.json</t>
         </is>
@@ -12878,7 +12974,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I85" s="35" t="inlineStr">
+      <c r="I85" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonCloudWatch/current/us-east-1/index.json</t>
         </is>
@@ -12923,7 +13019,7 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="I86" s="35" t="inlineStr">
+      <c r="I86" s="37" t="inlineStr">
         <is>
           <t>https://pricing.us-east-1.amazonaws.com/offers/v1.0/aws/AmazonCloudWatch/current/eu-south-2/index.json</t>
         </is>

</xml_diff>